<commit_message>
docs: add fuzzy Tahani method testing documentation and update Excel calculation dataset
</commit_message>
<xml_diff>
--- a/fuzzy.xlsx
+++ b/fuzzy.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TA\cabai\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TA\git ta\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8D782FE3-B346-4F8C-A59A-291E82C9228B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6D2CEB4-EBD7-423C-BDAE-C07BB0031FD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A7089781-A716-412D-87ED-AB088FC0AD4E}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
   <si>
     <t>No</t>
   </si>
@@ -84,12 +84,6 @@
   </si>
   <si>
     <t>Basah</t>
-  </si>
-  <si>
-    <t>OFF</t>
-  </si>
-  <si>
-    <t>ON</t>
   </si>
   <si>
     <t>25/6/2026 13:24</t>
@@ -176,10 +170,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -527,8 +522,9 @@
     <col min="8" max="8" width="5.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.140625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="6.5703125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="8" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="6.5703125" bestFit="1" customWidth="1"/>
@@ -559,31 +555,31 @@
         <v>12</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I1" s="2" t="s">
         <v>5</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>13</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="M1" s="2" t="s">
         <v>6</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="P1" s="2" t="s">
         <v>14</v>
@@ -627,58 +623,76 @@
         <v>79</v>
       </c>
       <c r="F2" s="1">
+        <f>IF(C2&lt;=5, 1, IF(C2&lt;=6, (6-C2)/(6-5), 0))</f>
         <v>1</v>
       </c>
       <c r="G2" s="1">
+        <f>IF(C2&lt;=5.5, 0, IF(C2&lt;=6, (C2-5.5)/(6-5.5),IF(C2&lt;=7, 1, IF(C2&lt;=7.5, (7.5-C2)/(7.5-7), 0))))</f>
         <v>0</v>
       </c>
       <c r="H2" s="1">
-        <v>0</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>12</v>
+        <f>IF(C2&lt;=7, 0, IF(C2&lt;=7.5, (C2-7)/(7.5-7), 1))</f>
+        <v>0</v>
+      </c>
+      <c r="I2" s="1" t="str">
+        <f>IF(AND(F2&gt;=G2,F2&gt;=H2),"Asam",IF(G2&gt;=H2,"Normal","Basa"))</f>
+        <v>Asam</v>
       </c>
       <c r="J2" s="1">
-        <v>0</v>
-      </c>
-      <c r="K2" s="1">
-        <v>0.15</v>
-      </c>
-      <c r="L2" s="1">
+        <f>IF(D2&lt;=24, 1, IF(D2&lt;=27, (27-D2)/(27-24), 0))</f>
+        <v>0</v>
+      </c>
+      <c r="K2" s="3">
+        <f>IF(D2&lt;=27,0,IF(D2&lt;=27,(D2-24)/(27-24),IF(D2&lt;=31,(31-D2)/(31-27),0)))</f>
+        <v>0.90000000000000036</v>
+      </c>
+      <c r="L2" s="3">
+        <f>IF(D2&lt;=27, 0, IF(D2&lt;=31, (D2-27)/(31-27), 1))</f>
+        <v>9.9999999999999645E-2</v>
+      </c>
+      <c r="M2" s="1" t="str">
+        <f>IF(AND(J2&gt;=K2,J2&gt;=L2),"Rendah",IF(K2&gt;=L2,"Sedang","Tinggi"))</f>
+        <v>Sedang</v>
+      </c>
+      <c r="N2" s="1">
+        <f>IF(E2&lt;=40, 1, IF(E2&lt;=50, (50-E2)/(50-40), 0))</f>
+        <v>0</v>
+      </c>
+      <c r="O2" s="1">
+        <f>IF(E2&lt;=40, 0, IF(E2&lt;=50, (E2-40)/(50-40),IF(E2&lt;=70, 1, IF(E2&lt;=80, (80-E2)/(80-70), 0))))</f>
         <v>0.1</v>
       </c>
-      <c r="M2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="N2" s="1">
-        <v>0</v>
-      </c>
-      <c r="O2" s="1">
-        <v>0.1</v>
-      </c>
       <c r="P2" s="1">
+        <f>IF(E2&lt;=70, 0, IF(E2&lt;=80, (E2-70)/(80-70), 1))</f>
         <v>0.9</v>
       </c>
-      <c r="Q2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="R2" s="1">
-        <v>0.1</v>
-      </c>
-      <c r="S2" s="1">
-        <v>0.1</v>
+      <c r="Q2" s="1" t="str">
+        <f>IF(AND(N2&gt;=O2,N2&gt;=P2),"Kering",IF(O2&gt;=P2,"Lembab","Basah"))</f>
+        <v>Basah</v>
+      </c>
+      <c r="R2" s="3">
+        <f>L2</f>
+        <v>9.9999999999999645E-2</v>
+      </c>
+      <c r="S2" s="3">
+        <f>MAX(N2, MIN(O2, L2))</f>
+        <v>9.9999999999999645E-2</v>
       </c>
       <c r="T2" s="1">
-        <v>1</v>
-      </c>
-      <c r="U2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="V2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="W2" s="1" t="s">
-        <v>16</v>
+        <f>F2</f>
+        <v>1</v>
+      </c>
+      <c r="U2" s="1" t="str">
+        <f>IF(R2&gt;0.5,"ON","OFF")</f>
+        <v>OFF</v>
+      </c>
+      <c r="V2" s="1" t="str">
+        <f>IF(S2&gt;0.4,"ON","OFF")</f>
+        <v>OFF</v>
+      </c>
+      <c r="W2" s="1" t="str">
+        <f>IF(T2&gt;0.4,"ON","OFF")</f>
+        <v>ON</v>
       </c>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.25">
@@ -686,7 +700,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C3" s="1">
         <v>5</v>
@@ -698,58 +712,76 @@
         <v>79</v>
       </c>
       <c r="F3" s="1">
+        <f t="shared" ref="F3:F6" si="0">IF(C3&lt;=5, 1, IF(C3&lt;=6, (6-C3)/(6-5), 0))</f>
         <v>1</v>
       </c>
       <c r="G3" s="1">
+        <f t="shared" ref="G3:G6" si="1">IF(C3&lt;=5.5, 0, IF(C3&lt;=6, (C3-5.5)/(6-5.5),IF(C3&lt;=7, 1, IF(C3&lt;=7.5, (7.5-C3)/(7.5-7), 0))))</f>
         <v>0</v>
       </c>
       <c r="H3" s="1">
-        <v>0</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>12</v>
+        <f t="shared" ref="H3:H6" si="2">IF(C3&lt;=7, 0, IF(C3&lt;=7.5, (C3-7)/(7.5-7), 1))</f>
+        <v>0</v>
+      </c>
+      <c r="I3" s="1" t="str">
+        <f t="shared" ref="I3:I6" si="3">IF(AND(F3&gt;=G3,F3&gt;=H3),"Asam",IF(G3&gt;=H3,"Normal","Basa"))</f>
+        <v>Asam</v>
       </c>
       <c r="J3" s="1">
-        <v>0</v>
-      </c>
-      <c r="K3" s="1">
-        <v>0.13</v>
-      </c>
-      <c r="L3" s="1">
-        <v>0.13</v>
-      </c>
-      <c r="M3" s="1" t="s">
-        <v>13</v>
+        <f t="shared" ref="J3:J6" si="4">IF(D3&lt;=24, 1, IF(D3&lt;=27, (27-D3)/(27-24), 0))</f>
+        <v>0</v>
+      </c>
+      <c r="K3" s="3">
+        <f t="shared" ref="K3:K6" si="5">IF(D3&lt;=27,0,IF(D3&lt;=27,(D3-24)/(27-24),IF(D3&lt;=31,(31-D3)/(31-27),0)))</f>
+        <v>0.875</v>
+      </c>
+      <c r="L3" s="3">
+        <f t="shared" ref="L3:L6" si="6">IF(D3&lt;=27, 0, IF(D3&lt;=31, (D3-27)/(31-27), 1))</f>
+        <v>0.125</v>
+      </c>
+      <c r="M3" s="1" t="str">
+        <f t="shared" ref="M3:M6" si="7">IF(AND(J3&gt;=K3,J3&gt;=L3),"Rendah",IF(K3&gt;=L3,"Sedang","Tinggi"))</f>
+        <v>Sedang</v>
       </c>
       <c r="N3" s="1">
+        <f t="shared" ref="N3:N6" si="8">IF(E3&lt;=40, 1, IF(E3&lt;=50, (50-E3)/(50-40), 0))</f>
         <v>0</v>
       </c>
       <c r="O3" s="1">
+        <f t="shared" ref="O3:O6" si="9">IF(E3&lt;=40, 0, IF(E3&lt;=50, (E3-40)/(50-40),IF(E3&lt;=70, 1, IF(E3&lt;=80, (80-E3)/(80-70), 0))))</f>
         <v>0.1</v>
       </c>
       <c r="P3" s="1">
+        <f t="shared" ref="P3:P6" si="10">IF(E3&lt;=70, 0, IF(E3&lt;=80, (E3-70)/(80-70), 1))</f>
         <v>0.9</v>
       </c>
-      <c r="Q3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="R3" s="1">
-        <v>0.13</v>
-      </c>
-      <c r="S3" s="1">
+      <c r="Q3" s="1" t="str">
+        <f t="shared" ref="Q3:Q6" si="11">IF(AND(N3&gt;=O3,N3&gt;=P3),"Kering",IF(O3&gt;=P3,"Lembab","Basah"))</f>
+        <v>Basah</v>
+      </c>
+      <c r="R3" s="3">
+        <f t="shared" ref="R3:R6" si="12">L3</f>
+        <v>0.125</v>
+      </c>
+      <c r="S3" s="3">
+        <f t="shared" ref="S3:S6" si="13">MAX(N3, MIN(O3, L3))</f>
         <v>0.1</v>
       </c>
       <c r="T3" s="1">
-        <v>1</v>
-      </c>
-      <c r="U3" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="V3" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="W3" s="1" t="s">
-        <v>16</v>
+        <f t="shared" ref="T3:T6" si="14">F3</f>
+        <v>1</v>
+      </c>
+      <c r="U3" s="1" t="str">
+        <f t="shared" ref="U3:U6" si="15">IF(R3&gt;0.5,"ON","OFF")</f>
+        <v>OFF</v>
+      </c>
+      <c r="V3" s="1" t="str">
+        <f t="shared" ref="V3:V6" si="16">IF(S3&gt;0.4,"ON","OFF")</f>
+        <v>OFF</v>
+      </c>
+      <c r="W3" s="1" t="str">
+        <f t="shared" ref="W3:W6" si="17">IF(T3&gt;0.4,"ON","OFF")</f>
+        <v>ON</v>
       </c>
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.25">
@@ -757,7 +789,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C4" s="1">
         <v>5</v>
@@ -769,58 +801,76 @@
         <v>78</v>
       </c>
       <c r="F4" s="1">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="G4" s="1">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="H4" s="1">
-        <v>0</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>12</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I4" s="1" t="str">
+        <f t="shared" si="3"/>
+        <v>Asam</v>
       </c>
       <c r="J4" s="1">
-        <v>0</v>
-      </c>
-      <c r="K4" s="1">
-        <v>0.13</v>
-      </c>
-      <c r="L4" s="1">
-        <v>0.13</v>
-      </c>
-      <c r="M4" s="1" t="s">
-        <v>13</v>
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="K4" s="3">
+        <f t="shared" si="5"/>
+        <v>0.875</v>
+      </c>
+      <c r="L4" s="3">
+        <f t="shared" si="6"/>
+        <v>0.125</v>
+      </c>
+      <c r="M4" s="1" t="str">
+        <f t="shared" si="7"/>
+        <v>Sedang</v>
       </c>
       <c r="N4" s="1">
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="O4" s="1">
+        <f t="shared" si="9"/>
         <v>0.2</v>
       </c>
       <c r="P4" s="1">
+        <f t="shared" si="10"/>
         <v>0.8</v>
       </c>
-      <c r="Q4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="R4" s="1">
-        <v>0.13</v>
-      </c>
-      <c r="S4" s="1">
-        <v>0.13</v>
+      <c r="Q4" s="1" t="str">
+        <f t="shared" si="11"/>
+        <v>Basah</v>
+      </c>
+      <c r="R4" s="3">
+        <f t="shared" si="12"/>
+        <v>0.125</v>
+      </c>
+      <c r="S4" s="3">
+        <f t="shared" si="13"/>
+        <v>0.125</v>
       </c>
       <c r="T4" s="1">
-        <v>1</v>
-      </c>
-      <c r="U4" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="V4" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="W4" s="1" t="s">
-        <v>16</v>
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="U4" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v>OFF</v>
+      </c>
+      <c r="V4" s="1" t="str">
+        <f t="shared" si="16"/>
+        <v>OFF</v>
+      </c>
+      <c r="W4" s="1" t="str">
+        <f t="shared" si="17"/>
+        <v>ON</v>
       </c>
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.25">
@@ -828,7 +878,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C5" s="1">
         <v>5</v>
@@ -840,58 +890,76 @@
         <v>79</v>
       </c>
       <c r="F5" s="1">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="G5" s="1">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="H5" s="1">
-        <v>0</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>12</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I5" s="1" t="str">
+        <f t="shared" si="3"/>
+        <v>Asam</v>
       </c>
       <c r="J5" s="1">
-        <v>0</v>
-      </c>
-      <c r="K5" s="1">
-        <v>0.15</v>
-      </c>
-      <c r="L5" s="1">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="K5" s="3">
+        <f t="shared" si="5"/>
+        <v>0.90000000000000036</v>
+      </c>
+      <c r="L5" s="3">
+        <f t="shared" si="6"/>
+        <v>9.9999999999999645E-2</v>
+      </c>
+      <c r="M5" s="1" t="str">
+        <f t="shared" si="7"/>
+        <v>Sedang</v>
+      </c>
+      <c r="N5" s="1">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="O5" s="1">
+        <f t="shared" si="9"/>
         <v>0.1</v>
       </c>
-      <c r="M5" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="N5" s="1">
-        <v>0</v>
-      </c>
-      <c r="O5" s="1">
-        <v>0.1</v>
-      </c>
       <c r="P5" s="1">
+        <f t="shared" si="10"/>
         <v>0.9</v>
       </c>
-      <c r="Q5" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="R5" s="1">
-        <v>0.1</v>
-      </c>
-      <c r="S5" s="1">
-        <v>0.1</v>
+      <c r="Q5" s="1" t="str">
+        <f t="shared" si="11"/>
+        <v>Basah</v>
+      </c>
+      <c r="R5" s="3">
+        <f t="shared" si="12"/>
+        <v>9.9999999999999645E-2</v>
+      </c>
+      <c r="S5" s="3">
+        <f t="shared" si="13"/>
+        <v>9.9999999999999645E-2</v>
       </c>
       <c r="T5" s="1">
-        <v>1</v>
-      </c>
-      <c r="U5" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="V5" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="W5" s="1" t="s">
-        <v>16</v>
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="U5" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v>OFF</v>
+      </c>
+      <c r="V5" s="1" t="str">
+        <f t="shared" si="16"/>
+        <v>OFF</v>
+      </c>
+      <c r="W5" s="1" t="str">
+        <f t="shared" si="17"/>
+        <v>ON</v>
       </c>
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.25">
@@ -899,7 +967,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C6" s="1">
         <v>5</v>
@@ -911,58 +979,76 @@
         <v>79</v>
       </c>
       <c r="F6" s="1">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="G6" s="1">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="H6" s="1">
-        <v>0</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>12</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I6" s="1" t="str">
+        <f t="shared" si="3"/>
+        <v>Asam</v>
       </c>
       <c r="J6" s="1">
-        <v>0</v>
-      </c>
-      <c r="K6" s="1">
-        <v>0.2</v>
-      </c>
-      <c r="L6" s="1">
-        <v>0.05</v>
-      </c>
-      <c r="M6" s="1" t="s">
-        <v>13</v>
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="K6" s="3">
+        <f t="shared" si="5"/>
+        <v>0.95000000000000018</v>
+      </c>
+      <c r="L6" s="3">
+        <f t="shared" si="6"/>
+        <v>4.9999999999999822E-2</v>
+      </c>
+      <c r="M6" s="1" t="str">
+        <f t="shared" si="7"/>
+        <v>Sedang</v>
       </c>
       <c r="N6" s="1">
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="O6" s="1">
+        <f t="shared" si="9"/>
         <v>0.1</v>
       </c>
       <c r="P6" s="1">
+        <f t="shared" si="10"/>
         <v>0.9</v>
       </c>
-      <c r="Q6" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="R6" s="1">
-        <v>0.05</v>
-      </c>
-      <c r="S6" s="1">
-        <v>0.05</v>
+      <c r="Q6" s="1" t="str">
+        <f t="shared" si="11"/>
+        <v>Basah</v>
+      </c>
+      <c r="R6" s="3">
+        <f t="shared" si="12"/>
+        <v>4.9999999999999822E-2</v>
+      </c>
+      <c r="S6" s="3">
+        <f t="shared" si="13"/>
+        <v>4.9999999999999822E-2</v>
       </c>
       <c r="T6" s="1">
-        <v>1</v>
-      </c>
-      <c r="U6" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="V6" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="W6" s="1" t="s">
-        <v>16</v>
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="U6" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v>OFF</v>
+      </c>
+      <c r="V6" s="1" t="str">
+        <f t="shared" si="16"/>
+        <v>OFF</v>
+      </c>
+      <c r="W6" s="1" t="str">
+        <f t="shared" si="17"/>
+        <v>ON</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: update fuzzy matching parameters in fuzzy.xlsx
</commit_message>
<xml_diff>
--- a/fuzzy.xlsx
+++ b/fuzzy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TA\git ta\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6D2CEB4-EBD7-423C-BDAE-C07BB0031FD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB3C31ED-72A7-4591-8B98-B06C9D4A2AB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A7089781-A716-412D-87ED-AB088FC0AD4E}"/>
   </bookViews>
@@ -622,7 +622,7 @@
       <c r="E2" s="1">
         <v>79</v>
       </c>
-      <c r="F2" s="1">
+      <c r="F2" s="3">
         <f>IF(C2&lt;=5, 1, IF(C2&lt;=6, (6-C2)/(6-5), 0))</f>
         <v>1</v>
       </c>
@@ -658,7 +658,7 @@
         <f>IF(E2&lt;=40, 1, IF(E2&lt;=50, (50-E2)/(50-40), 0))</f>
         <v>0</v>
       </c>
-      <c r="O2" s="1">
+      <c r="O2" s="3">
         <f>IF(E2&lt;=40, 0, IF(E2&lt;=50, (E2-40)/(50-40),IF(E2&lt;=70, 1, IF(E2&lt;=80, (80-E2)/(80-70), 0))))</f>
         <v>0.1</v>
       </c>
@@ -678,7 +678,7 @@
         <f>MAX(N2, MIN(O2, L2))</f>
         <v>9.9999999999999645E-2</v>
       </c>
-      <c r="T2" s="1">
+      <c r="T2" s="3">
         <f>F2</f>
         <v>1</v>
       </c>
@@ -711,7 +711,7 @@
       <c r="E3" s="1">
         <v>79</v>
       </c>
-      <c r="F3" s="1">
+      <c r="F3" s="3">
         <f t="shared" ref="F3:F6" si="0">IF(C3&lt;=5, 1, IF(C3&lt;=6, (6-C3)/(6-5), 0))</f>
         <v>1</v>
       </c>
@@ -747,7 +747,7 @@
         <f t="shared" ref="N3:N6" si="8">IF(E3&lt;=40, 1, IF(E3&lt;=50, (50-E3)/(50-40), 0))</f>
         <v>0</v>
       </c>
-      <c r="O3" s="1">
+      <c r="O3" s="3">
         <f t="shared" ref="O3:O6" si="9">IF(E3&lt;=40, 0, IF(E3&lt;=50, (E3-40)/(50-40),IF(E3&lt;=70, 1, IF(E3&lt;=80, (80-E3)/(80-70), 0))))</f>
         <v>0.1</v>
       </c>
@@ -767,7 +767,7 @@
         <f t="shared" ref="S3:S6" si="13">MAX(N3, MIN(O3, L3))</f>
         <v>0.1</v>
       </c>
-      <c r="T3" s="1">
+      <c r="T3" s="3">
         <f t="shared" ref="T3:T6" si="14">F3</f>
         <v>1</v>
       </c>
@@ -800,7 +800,7 @@
       <c r="E4" s="1">
         <v>78</v>
       </c>
-      <c r="F4" s="1">
+      <c r="F4" s="3">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
@@ -836,7 +836,7 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="O4" s="1">
+      <c r="O4" s="3">
         <f t="shared" si="9"/>
         <v>0.2</v>
       </c>
@@ -856,7 +856,7 @@
         <f t="shared" si="13"/>
         <v>0.125</v>
       </c>
-      <c r="T4" s="1">
+      <c r="T4" s="3">
         <f t="shared" si="14"/>
         <v>1</v>
       </c>
@@ -889,7 +889,7 @@
       <c r="E5" s="1">
         <v>79</v>
       </c>
-      <c r="F5" s="1">
+      <c r="F5" s="3">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
@@ -925,7 +925,7 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="O5" s="1">
+      <c r="O5" s="3">
         <f t="shared" si="9"/>
         <v>0.1</v>
       </c>
@@ -945,7 +945,7 @@
         <f t="shared" si="13"/>
         <v>9.9999999999999645E-2</v>
       </c>
-      <c r="T5" s="1">
+      <c r="T5" s="3">
         <f t="shared" si="14"/>
         <v>1</v>
       </c>
@@ -978,7 +978,7 @@
       <c r="E6" s="1">
         <v>79</v>
       </c>
-      <c r="F6" s="1">
+      <c r="F6" s="3">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
@@ -1014,7 +1014,7 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="O6" s="1">
+      <c r="O6" s="3">
         <f t="shared" si="9"/>
         <v>0.1</v>
       </c>
@@ -1034,7 +1034,7 @@
         <f t="shared" si="13"/>
         <v>4.9999999999999822E-2</v>
       </c>
-      <c r="T6" s="1">
+      <c r="T6" s="3">
         <f t="shared" si="14"/>
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
feat: add documentation for pump timing logic and update fuzzy configuration spreadsheet
</commit_message>
<xml_diff>
--- a/fuzzy.xlsx
+++ b/fuzzy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TA\git ta\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB3C31ED-72A7-4591-8B98-B06C9D4A2AB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F061460-705A-4539-A53A-C247F0CEFA21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A7089781-A716-412D-87ED-AB088FC0AD4E}"/>
   </bookViews>
@@ -172,9 +172,15 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -509,6 +515,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB814642-682D-4D33-90CA-80D617FFCD53}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:W6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -521,7 +530,7 @@
     <col min="7" max="7" width="7.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="5.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7.7109375" customWidth="1"/>
     <col min="11" max="11" width="8.140625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="6.28515625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -536,109 +545,109 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="P1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="Q1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="R1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="S1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="T1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="U1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="V1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="W1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A2" s="1">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1" t="s">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2" s="2">
         <v>5</v>
       </c>
-      <c r="D2" s="1">
+      <c r="D2" s="2">
         <v>27.4</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>79</v>
       </c>
       <c r="F2" s="3">
         <f>IF(C2&lt;=5, 1, IF(C2&lt;=6, (6-C2)/(6-5), 0))</f>
         <v>1</v>
       </c>
-      <c r="G2" s="1">
+      <c r="G2" s="2">
         <f>IF(C2&lt;=5.5, 0, IF(C2&lt;=6, (C2-5.5)/(6-5.5),IF(C2&lt;=7, 1, IF(C2&lt;=7.5, (7.5-C2)/(7.5-7), 0))))</f>
         <v>0</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <f>IF(C2&lt;=7, 0, IF(C2&lt;=7.5, (C2-7)/(7.5-7), 1))</f>
         <v>0</v>
       </c>
-      <c r="I2" s="1" t="str">
+      <c r="I2" s="2" t="str">
         <f>IF(AND(F2&gt;=G2,F2&gt;=H2),"Asam",IF(G2&gt;=H2,"Normal","Basa"))</f>
         <v>Asam</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <f>IF(D2&lt;=24, 1, IF(D2&lt;=27, (27-D2)/(27-24), 0))</f>
         <v>0</v>
       </c>
@@ -650,11 +659,11 @@
         <f>IF(D2&lt;=27, 0, IF(D2&lt;=31, (D2-27)/(31-27), 1))</f>
         <v>9.9999999999999645E-2</v>
       </c>
-      <c r="M2" s="1" t="str">
+      <c r="M2" s="2" t="str">
         <f>IF(AND(J2&gt;=K2,J2&gt;=L2),"Rendah",IF(K2&gt;=L2,"Sedang","Tinggi"))</f>
         <v>Sedang</v>
       </c>
-      <c r="N2" s="1">
+      <c r="N2" s="2">
         <f>IF(E2&lt;=40, 1, IF(E2&lt;=50, (50-E2)/(50-40), 0))</f>
         <v>0</v>
       </c>
@@ -662,11 +671,11 @@
         <f>IF(E2&lt;=40, 0, IF(E2&lt;=50, (E2-40)/(50-40),IF(E2&lt;=70, 1, IF(E2&lt;=80, (80-E2)/(80-70), 0))))</f>
         <v>0.1</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <f>IF(E2&lt;=70, 0, IF(E2&lt;=80, (E2-70)/(80-70), 1))</f>
         <v>0.9</v>
       </c>
-      <c r="Q2" s="1" t="str">
+      <c r="Q2" s="2" t="str">
         <f>IF(AND(N2&gt;=O2,N2&gt;=P2),"Kering",IF(O2&gt;=P2,"Lembab","Basah"))</f>
         <v>Basah</v>
       </c>
@@ -682,376 +691,377 @@
         <f>F2</f>
         <v>1</v>
       </c>
-      <c r="U2" s="1" t="str">
+      <c r="U2" s="2" t="str">
         <f>IF(R2&gt;0.5,"ON","OFF")</f>
         <v>OFF</v>
       </c>
-      <c r="V2" s="1" t="str">
+      <c r="V2" s="2" t="str">
         <f>IF(S2&gt;0.4,"ON","OFF")</f>
         <v>OFF</v>
       </c>
-      <c r="W2" s="1" t="str">
+      <c r="W2" s="2" t="str">
         <f>IF(T2&gt;0.4,"ON","OFF")</f>
         <v>ON</v>
       </c>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3" s="2">
         <v>5</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3" s="2">
         <v>27.5</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>79</v>
       </c>
       <c r="F3" s="3">
         <f t="shared" ref="F3:F6" si="0">IF(C3&lt;=5, 1, IF(C3&lt;=6, (6-C3)/(6-5), 0))</f>
         <v>1</v>
       </c>
-      <c r="G3" s="1">
+      <c r="G3" s="2">
         <f t="shared" ref="G3:G6" si="1">IF(C3&lt;=5.5, 0, IF(C3&lt;=6, (C3-5.5)/(6-5.5),IF(C3&lt;=7, 1, IF(C3&lt;=7.5, (7.5-C3)/(7.5-7), 0))))</f>
         <v>0</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <f t="shared" ref="H3:H6" si="2">IF(C3&lt;=7, 0, IF(C3&lt;=7.5, (C3-7)/(7.5-7), 1))</f>
         <v>0</v>
       </c>
-      <c r="I3" s="1" t="str">
+      <c r="I3" s="2" t="str">
         <f t="shared" ref="I3:I6" si="3">IF(AND(F3&gt;=G3,F3&gt;=H3),"Asam",IF(G3&gt;=H3,"Normal","Basa"))</f>
         <v>Asam</v>
       </c>
-      <c r="J3" s="1">
-        <f t="shared" ref="J3:J6" si="4">IF(D3&lt;=24, 1, IF(D3&lt;=27, (27-D3)/(27-24), 0))</f>
+      <c r="J3" s="2">
+        <f>IF(D3&lt;=24, 1, IF(D3&lt;=27, (27-D3)/(27-24), 0))</f>
         <v>0</v>
       </c>
       <c r="K3" s="3">
-        <f t="shared" ref="K3:K6" si="5">IF(D3&lt;=27,0,IF(D3&lt;=27,(D3-24)/(27-24),IF(D3&lt;=31,(31-D3)/(31-27),0)))</f>
+        <f>IF(D3&lt;=27,0,IF(D3&lt;=27,(D3-24)/(27-24),IF(D3&lt;=31,(31-D3)/(31-27),0)))</f>
         <v>0.875</v>
       </c>
       <c r="L3" s="3">
-        <f t="shared" ref="L3:L6" si="6">IF(D3&lt;=27, 0, IF(D3&lt;=31, (D3-27)/(31-27), 1))</f>
+        <f>IF(D3&lt;=27, 0, IF(D3&lt;=31, (D3-27)/(31-27), 1))</f>
         <v>0.125</v>
       </c>
-      <c r="M3" s="1" t="str">
-        <f t="shared" ref="M3:M6" si="7">IF(AND(J3&gt;=K3,J3&gt;=L3),"Rendah",IF(K3&gt;=L3,"Sedang","Tinggi"))</f>
+      <c r="M3" s="2" t="str">
+        <f>IF(AND(J3&gt;=K3,J3&gt;=L3),"Rendah",IF(K3&gt;=L3,"Sedang","Tinggi"))</f>
         <v>Sedang</v>
       </c>
-      <c r="N3" s="1">
-        <f t="shared" ref="N3:N6" si="8">IF(E3&lt;=40, 1, IF(E3&lt;=50, (50-E3)/(50-40), 0))</f>
+      <c r="N3" s="2">
+        <f>IF(E3&lt;=40, 1, IF(E3&lt;=50, (50-E3)/(50-40), 0))</f>
         <v>0</v>
       </c>
       <c r="O3" s="3">
-        <f t="shared" ref="O3:O6" si="9">IF(E3&lt;=40, 0, IF(E3&lt;=50, (E3-40)/(50-40),IF(E3&lt;=70, 1, IF(E3&lt;=80, (80-E3)/(80-70), 0))))</f>
+        <f>IF(E3&lt;=40, 0, IF(E3&lt;=50, (E3-40)/(50-40),IF(E3&lt;=70, 1, IF(E3&lt;=80, (80-E3)/(80-70), 0))))</f>
         <v>0.1</v>
       </c>
-      <c r="P3" s="1">
-        <f t="shared" ref="P3:P6" si="10">IF(E3&lt;=70, 0, IF(E3&lt;=80, (E3-70)/(80-70), 1))</f>
+      <c r="P3" s="2">
+        <f>IF(E3&lt;=70, 0, IF(E3&lt;=80, (E3-70)/(80-70), 1))</f>
         <v>0.9</v>
       </c>
-      <c r="Q3" s="1" t="str">
-        <f t="shared" ref="Q3:Q6" si="11">IF(AND(N3&gt;=O3,N3&gt;=P3),"Kering",IF(O3&gt;=P3,"Lembab","Basah"))</f>
+      <c r="Q3" s="2" t="str">
+        <f>IF(AND(N3&gt;=O3,N3&gt;=P3),"Kering",IF(O3&gt;=P3,"Lembab","Basah"))</f>
         <v>Basah</v>
       </c>
       <c r="R3" s="3">
-        <f t="shared" ref="R3:R6" si="12">L3</f>
+        <f>L3</f>
         <v>0.125</v>
       </c>
       <c r="S3" s="3">
-        <f t="shared" ref="S3:S6" si="13">MAX(N3, MIN(O3, L3))</f>
+        <f>MAX(N3, MIN(O3, L3))</f>
         <v>0.1</v>
       </c>
       <c r="T3" s="3">
-        <f t="shared" ref="T3:T6" si="14">F3</f>
-        <v>1</v>
-      </c>
-      <c r="U3" s="1" t="str">
-        <f t="shared" ref="U3:U6" si="15">IF(R3&gt;0.5,"ON","OFF")</f>
+        <f t="shared" ref="T3:T6" si="4">F3</f>
+        <v>1</v>
+      </c>
+      <c r="U3" s="2" t="str">
+        <f t="shared" ref="U3:U6" si="5">IF(R3&gt;0.5,"ON","OFF")</f>
         <v>OFF</v>
       </c>
-      <c r="V3" s="1" t="str">
-        <f t="shared" ref="V3:V6" si="16">IF(S3&gt;0.4,"ON","OFF")</f>
+      <c r="V3" s="2" t="str">
+        <f t="shared" ref="V3:V6" si="6">IF(S3&gt;0.4,"ON","OFF")</f>
         <v>OFF</v>
       </c>
-      <c r="W3" s="1" t="str">
-        <f t="shared" ref="W3:W6" si="17">IF(T3&gt;0.4,"ON","OFF")</f>
+      <c r="W3" s="2" t="str">
+        <f t="shared" ref="W3:W6" si="7">IF(T3&gt;0.4,"ON","OFF")</f>
         <v>ON</v>
       </c>
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>3</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" s="2">
         <v>5</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="2">
         <v>27.5</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>78</v>
       </c>
       <c r="F4" s="3">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="G4" s="1">
+      <c r="G4" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="I4" s="1" t="str">
+      <c r="I4" s="2" t="str">
         <f t="shared" si="3"/>
         <v>Asam</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
+        <f>IF(D4&lt;=24, 1, IF(D4&lt;=27, (27-D4)/(27-24), 0))</f>
+        <v>0</v>
+      </c>
+      <c r="K4" s="3">
+        <f>IF(D4&lt;=27,0,IF(D4&lt;=27,(D4-24)/(27-24),IF(D4&lt;=31,(31-D4)/(31-27),0)))</f>
+        <v>0.875</v>
+      </c>
+      <c r="L4" s="3">
+        <f>IF(D4&lt;=27, 0, IF(D4&lt;=31, (D4-27)/(31-27), 1))</f>
+        <v>0.125</v>
+      </c>
+      <c r="M4" s="2" t="str">
+        <f>IF(AND(J4&gt;=K4,J4&gt;=L4),"Rendah",IF(K4&gt;=L4,"Sedang","Tinggi"))</f>
+        <v>Sedang</v>
+      </c>
+      <c r="N4" s="2">
+        <f>IF(E4&lt;=40, 1, IF(E4&lt;=50, (50-E4)/(50-40), 0))</f>
+        <v>0</v>
+      </c>
+      <c r="O4" s="3">
+        <f>IF(E4&lt;=40, 0, IF(E4&lt;=50, (E4-40)/(50-40),IF(E4&lt;=70, 1, IF(E4&lt;=80, (80-E4)/(80-70), 0))))</f>
+        <v>0.2</v>
+      </c>
+      <c r="P4" s="2">
+        <f>IF(E4&lt;=70, 0, IF(E4&lt;=80, (E4-70)/(80-70), 1))</f>
+        <v>0.8</v>
+      </c>
+      <c r="Q4" s="2" t="str">
+        <f>IF(AND(N4&gt;=O4,N4&gt;=P4),"Kering",IF(O4&gt;=P4,"Lembab","Basah"))</f>
+        <v>Basah</v>
+      </c>
+      <c r="R4" s="3">
+        <f>L4</f>
+        <v>0.125</v>
+      </c>
+      <c r="S4" s="3">
+        <f>MAX(N4, MIN(O4, L4))</f>
+        <v>0.125</v>
+      </c>
+      <c r="T4" s="3">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="K4" s="3">
+        <v>1</v>
+      </c>
+      <c r="U4" s="2" t="str">
         <f t="shared" si="5"/>
-        <v>0.875</v>
-      </c>
-      <c r="L4" s="3">
+        <v>OFF</v>
+      </c>
+      <c r="V4" s="2" t="str">
         <f t="shared" si="6"/>
-        <v>0.125</v>
-      </c>
-      <c r="M4" s="1" t="str">
+        <v>OFF</v>
+      </c>
+      <c r="W4" s="2" t="str">
         <f t="shared" si="7"/>
-        <v>Sedang</v>
-      </c>
-      <c r="N4" s="1">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="O4" s="3">
-        <f t="shared" si="9"/>
-        <v>0.2</v>
-      </c>
-      <c r="P4" s="1">
-        <f t="shared" si="10"/>
-        <v>0.8</v>
-      </c>
-      <c r="Q4" s="1" t="str">
-        <f t="shared" si="11"/>
-        <v>Basah</v>
-      </c>
-      <c r="R4" s="3">
-        <f t="shared" si="12"/>
-        <v>0.125</v>
-      </c>
-      <c r="S4" s="3">
-        <f t="shared" si="13"/>
-        <v>0.125</v>
-      </c>
-      <c r="T4" s="3">
-        <f t="shared" si="14"/>
-        <v>1</v>
-      </c>
-      <c r="U4" s="1" t="str">
-        <f t="shared" si="15"/>
-        <v>OFF</v>
-      </c>
-      <c r="V4" s="1" t="str">
-        <f t="shared" si="16"/>
-        <v>OFF</v>
-      </c>
-      <c r="W4" s="1" t="str">
-        <f t="shared" si="17"/>
         <v>ON</v>
       </c>
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>4</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" s="2">
         <v>5</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="2">
         <v>27.4</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>79</v>
       </c>
       <c r="F5" s="3">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="G5" s="1">
+      <c r="G5" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="I5" s="1" t="str">
+      <c r="I5" s="2" t="str">
         <f t="shared" si="3"/>
         <v>Asam</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
+        <f>IF(D5&lt;=24, 1, IF(D5&lt;=27, (27-D5)/(27-24), 0))</f>
+        <v>0</v>
+      </c>
+      <c r="K5" s="3">
+        <f>IF(D5&lt;=27,0,IF(D5&lt;=27,(D5-24)/(27-24),IF(D5&lt;=31,(31-D5)/(31-27),0)))</f>
+        <v>0.90000000000000036</v>
+      </c>
+      <c r="L5" s="3">
+        <f>IF(D5&lt;=27, 0, IF(D5&lt;=31, (D5-27)/(31-27), 1))</f>
+        <v>9.9999999999999645E-2</v>
+      </c>
+      <c r="M5" s="2" t="str">
+        <f>IF(AND(J5&gt;=K5,J5&gt;=L5),"Rendah",IF(K5&gt;=L5,"Sedang","Tinggi"))</f>
+        <v>Sedang</v>
+      </c>
+      <c r="N5" s="2">
+        <f>IF(E5&lt;=40, 1, IF(E5&lt;=50, (50-E5)/(50-40), 0))</f>
+        <v>0</v>
+      </c>
+      <c r="O5" s="3">
+        <f>IF(E5&lt;=40, 0, IF(E5&lt;=50, (E5-40)/(50-40),IF(E5&lt;=70, 1, IF(E5&lt;=80, (80-E5)/(80-70), 0))))</f>
+        <v>0.1</v>
+      </c>
+      <c r="P5" s="2">
+        <f>IF(E5&lt;=70, 0, IF(E5&lt;=80, (E5-70)/(80-70), 1))</f>
+        <v>0.9</v>
+      </c>
+      <c r="Q5" s="2" t="str">
+        <f>IF(AND(N5&gt;=O5,N5&gt;=P5),"Kering",IF(O5&gt;=P5,"Lembab","Basah"))</f>
+        <v>Basah</v>
+      </c>
+      <c r="R5" s="3">
+        <f>L5</f>
+        <v>9.9999999999999645E-2</v>
+      </c>
+      <c r="S5" s="3">
+        <f>MAX(N5, MIN(O5, L5))</f>
+        <v>9.9999999999999645E-2</v>
+      </c>
+      <c r="T5" s="3">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="K5" s="3">
+        <v>1</v>
+      </c>
+      <c r="U5" s="2" t="str">
         <f t="shared" si="5"/>
-        <v>0.90000000000000036</v>
-      </c>
-      <c r="L5" s="3">
+        <v>OFF</v>
+      </c>
+      <c r="V5" s="2" t="str">
         <f t="shared" si="6"/>
-        <v>9.9999999999999645E-2</v>
-      </c>
-      <c r="M5" s="1" t="str">
+        <v>OFF</v>
+      </c>
+      <c r="W5" s="2" t="str">
         <f t="shared" si="7"/>
-        <v>Sedang</v>
-      </c>
-      <c r="N5" s="1">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="O5" s="3">
-        <f t="shared" si="9"/>
-        <v>0.1</v>
-      </c>
-      <c r="P5" s="1">
-        <f t="shared" si="10"/>
-        <v>0.9</v>
-      </c>
-      <c r="Q5" s="1" t="str">
-        <f t="shared" si="11"/>
-        <v>Basah</v>
-      </c>
-      <c r="R5" s="3">
-        <f t="shared" si="12"/>
-        <v>9.9999999999999645E-2</v>
-      </c>
-      <c r="S5" s="3">
-        <f t="shared" si="13"/>
-        <v>9.9999999999999645E-2</v>
-      </c>
-      <c r="T5" s="3">
-        <f t="shared" si="14"/>
-        <v>1</v>
-      </c>
-      <c r="U5" s="1" t="str">
-        <f t="shared" si="15"/>
-        <v>OFF</v>
-      </c>
-      <c r="V5" s="1" t="str">
-        <f t="shared" si="16"/>
-        <v>OFF</v>
-      </c>
-      <c r="W5" s="1" t="str">
-        <f t="shared" si="17"/>
         <v>ON</v>
       </c>
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>5</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C6" s="2">
         <v>5</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D6" s="2">
         <v>27.2</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>79</v>
       </c>
       <c r="F6" s="3">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="G6" s="1">
+      <c r="G6" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="I6" s="1" t="str">
+      <c r="I6" s="2" t="str">
         <f t="shared" si="3"/>
         <v>Asam</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
+        <f>IF(D6&lt;=24, 1, IF(D6&lt;=27, (27-D6)/(27-24), 0))</f>
+        <v>0</v>
+      </c>
+      <c r="K6" s="3">
+        <f>IF(D6&lt;=27,0,IF(D6&lt;=27,(D6-24)/(27-24),IF(D6&lt;=31,(31-D6)/(31-27),0)))</f>
+        <v>0.95000000000000018</v>
+      </c>
+      <c r="L6" s="3">
+        <f>IF(D6&lt;=27, 0, IF(D6&lt;=31, (D6-27)/(31-27), 1))</f>
+        <v>4.9999999999999822E-2</v>
+      </c>
+      <c r="M6" s="2" t="str">
+        <f>IF(AND(J6&gt;=K6,J6&gt;=L6),"Rendah",IF(K6&gt;=L6,"Sedang","Tinggi"))</f>
+        <v>Sedang</v>
+      </c>
+      <c r="N6" s="2">
+        <f>IF(E6&lt;=40, 1, IF(E6&lt;=50, (50-E6)/(50-40), 0))</f>
+        <v>0</v>
+      </c>
+      <c r="O6" s="3">
+        <f>IF(E6&lt;=40, 0, IF(E6&lt;=50, (E6-40)/(50-40),IF(E6&lt;=70, 1, IF(E6&lt;=80, (80-E6)/(80-70), 0))))</f>
+        <v>0.1</v>
+      </c>
+      <c r="P6" s="2">
+        <f>IF(E6&lt;=70, 0, IF(E6&lt;=80, (E6-70)/(80-70), 1))</f>
+        <v>0.9</v>
+      </c>
+      <c r="Q6" s="2" t="str">
+        <f>IF(AND(N6&gt;=O6,N6&gt;=P6),"Kering",IF(O6&gt;=P6,"Lembab","Basah"))</f>
+        <v>Basah</v>
+      </c>
+      <c r="R6" s="3">
+        <f>L6</f>
+        <v>4.9999999999999822E-2</v>
+      </c>
+      <c r="S6" s="3">
+        <f>MAX(N6, MIN(O6, L6))</f>
+        <v>4.9999999999999822E-2</v>
+      </c>
+      <c r="T6" s="3">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="K6" s="3">
+        <v>1</v>
+      </c>
+      <c r="U6" s="2" t="str">
         <f t="shared" si="5"/>
-        <v>0.95000000000000018</v>
-      </c>
-      <c r="L6" s="3">
+        <v>OFF</v>
+      </c>
+      <c r="V6" s="2" t="str">
         <f t="shared" si="6"/>
-        <v>4.9999999999999822E-2</v>
-      </c>
-      <c r="M6" s="1" t="str">
+        <v>OFF</v>
+      </c>
+      <c r="W6" s="2" t="str">
         <f t="shared" si="7"/>
-        <v>Sedang</v>
-      </c>
-      <c r="N6" s="1">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="O6" s="3">
-        <f t="shared" si="9"/>
-        <v>0.1</v>
-      </c>
-      <c r="P6" s="1">
-        <f t="shared" si="10"/>
-        <v>0.9</v>
-      </c>
-      <c r="Q6" s="1" t="str">
-        <f t="shared" si="11"/>
-        <v>Basah</v>
-      </c>
-      <c r="R6" s="3">
-        <f t="shared" si="12"/>
-        <v>4.9999999999999822E-2</v>
-      </c>
-      <c r="S6" s="3">
-        <f t="shared" si="13"/>
-        <v>4.9999999999999822E-2</v>
-      </c>
-      <c r="T6" s="3">
-        <f t="shared" si="14"/>
-        <v>1</v>
-      </c>
-      <c r="U6" s="1" t="str">
-        <f t="shared" si="15"/>
-        <v>OFF</v>
-      </c>
-      <c r="V6" s="1" t="str">
-        <f t="shared" si="16"/>
-        <v>OFF</v>
-      </c>
-      <c r="W6" s="1" t="str">
-        <f t="shared" si="17"/>
         <v>ON</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup scale="69" orientation="landscape" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: update pengujian_fuzzy_tahani.md with extreme scenario testing results and add new data to fuzzy.xlsx
</commit_message>
<xml_diff>
--- a/fuzzy.xlsx
+++ b/fuzzy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TA\git ta\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F061460-705A-4539-A53A-C247F0CEFA21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A268B935-A2EC-4499-B916-19E0B813EA95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A7089781-A716-412D-87ED-AB088FC0AD4E}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="29">
   <si>
     <t>No</t>
   </si>
@@ -74,9 +74,6 @@
     <t>PompaPH</t>
   </si>
   <si>
-    <t>25/6/2026 13:25</t>
-  </si>
-  <si>
     <t>Asam</t>
   </si>
   <si>
@@ -86,18 +83,6 @@
     <t>Basah</t>
   </si>
   <si>
-    <t>25/6/2026 13:24</t>
-  </si>
-  <si>
-    <t>25/6/2026 13:23</t>
-  </si>
-  <si>
-    <t>25/6/2026 13:22</t>
-  </si>
-  <si>
-    <t>25/6/2026 13:21</t>
-  </si>
-  <si>
     <t>Normal</t>
   </si>
   <si>
@@ -114,12 +99,42 @@
   </si>
   <si>
     <t>Lembab</t>
+  </si>
+  <si>
+    <t>Variabel</t>
+  </si>
+  <si>
+    <t>Himpunan</t>
+  </si>
+  <si>
+    <t>Bawah</t>
+  </si>
+  <si>
+    <t>Tengah</t>
+  </si>
+  <si>
+    <t>Atas</t>
+  </si>
+  <si>
+    <t>pH Tanah</t>
+  </si>
+  <si>
+    <t>Suhu Udara</t>
+  </si>
+  <si>
+    <t>Kelembapan</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Tanah</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="176" formatCode="0.0"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -170,7 +185,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -179,6 +194,14 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -518,7 +541,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:W6"/>
+  <dimension ref="F1:W17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.5703125" bestFit="1" customWidth="1"/>
@@ -527,16 +550,16 @@
     <col min="4" max="4" width="5.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="6.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.85546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="5.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7.7109375" customWidth="1"/>
+    <col min="10" max="10" width="7.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="8.140625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="6.28515625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.28515625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="8" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="7.42578125" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="6" bestFit="1" customWidth="1"/>
     <col min="19" max="20" width="9.7109375" bestFit="1" customWidth="1"/>
@@ -544,54 +567,39 @@
     <col min="22" max="23" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
+    <row r="1" spans="6:23" x14ac:dyDescent="0.25">
       <c r="F1" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>5</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="Q1" s="1" t="s">
         <v>7</v>
@@ -615,81 +623,66 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
+    <row r="2" spans="6:23" x14ac:dyDescent="0.25">
+      <c r="F2" s="3">
+        <f>IF(H9&lt;=5, 1, IF(H9&lt;=6, (6-H9)/(6-5), 0))</f>
+        <v>0</v>
+      </c>
+      <c r="G2" s="2">
+        <f>IF(H9&lt;=5.5, 0, IF(H9&lt;=6, (H9-5.5)/(6-5.5),IF(H9&lt;=7, 1, IF(H9&lt;=7.5, (7.5-H9)/(7.5-7), 0))))</f>
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" s="2">
-        <v>5</v>
-      </c>
-      <c r="D2" s="2">
-        <v>27.4</v>
-      </c>
-      <c r="E2" s="2">
-        <v>79</v>
-      </c>
-      <c r="F2" s="3">
-        <f>IF(C2&lt;=5, 1, IF(C2&lt;=6, (6-C2)/(6-5), 0))</f>
-        <v>1</v>
-      </c>
-      <c r="G2" s="2">
-        <f>IF(C2&lt;=5.5, 0, IF(C2&lt;=6, (C2-5.5)/(6-5.5),IF(C2&lt;=7, 1, IF(C2&lt;=7.5, (7.5-C2)/(7.5-7), 0))))</f>
-        <v>0</v>
-      </c>
       <c r="H2" s="2">
-        <f>IF(C2&lt;=7, 0, IF(C2&lt;=7.5, (C2-7)/(7.5-7), 1))</f>
+        <f>IF(H9&lt;=7, 0, IF(H9&lt;=7.5, (H9-7)/(7.5-7), 1))</f>
         <v>0</v>
       </c>
       <c r="I2" s="2" t="str">
         <f>IF(AND(F2&gt;=G2,F2&gt;=H2),"Asam",IF(G2&gt;=H2,"Normal","Basa"))</f>
-        <v>Asam</v>
+        <v>Normal</v>
       </c>
       <c r="J2" s="2">
-        <f>IF(D2&lt;=24, 1, IF(D2&lt;=27, (27-D2)/(27-24), 0))</f>
-        <v>0</v>
+        <f>IF(I9&lt;=24, 1, IF(I9&lt;=27, (27-I9)/(27-24), 0))</f>
+        <v>1</v>
       </c>
       <c r="K2" s="3">
-        <f>IF(D2&lt;=27,0,IF(D2&lt;=27,(D2-24)/(27-24),IF(D2&lt;=31,(31-D2)/(31-27),0)))</f>
-        <v>0.90000000000000036</v>
+        <f>IF(I9&lt;=27,0,IF(I9&lt;=27,(I9-24)/(27-24),IF(I9&lt;=31,(31-I9)/(31-27),0)))</f>
+        <v>0</v>
       </c>
       <c r="L2" s="3">
-        <f>IF(D2&lt;=27, 0, IF(D2&lt;=31, (D2-27)/(31-27), 1))</f>
-        <v>9.9999999999999645E-2</v>
+        <f>IF(I9&lt;=27, 0, IF(I9&lt;=31, (I9-27)/(31-27), 1))</f>
+        <v>0</v>
       </c>
       <c r="M2" s="2" t="str">
         <f>IF(AND(J2&gt;=K2,J2&gt;=L2),"Rendah",IF(K2&gt;=L2,"Sedang","Tinggi"))</f>
-        <v>Sedang</v>
+        <v>Rendah</v>
       </c>
       <c r="N2" s="2">
-        <f>IF(E2&lt;=40, 1, IF(E2&lt;=50, (50-E2)/(50-40), 0))</f>
+        <f>IF(J9&lt;=40, 1, IF(J9&lt;=50, (50-J9)/(50-40), 0))</f>
         <v>0</v>
       </c>
       <c r="O2" s="3">
-        <f>IF(E2&lt;=40, 0, IF(E2&lt;=50, (E2-40)/(50-40),IF(E2&lt;=70, 1, IF(E2&lt;=80, (80-E2)/(80-70), 0))))</f>
-        <v>0.1</v>
+        <f>IF(J9&lt;=40, 0, IF(J9&lt;=50, (J9-40)/(50-40),IF(J9&lt;=70, 1, IF(J9&lt;=80, (80-J9)/(80-70), 0))))</f>
+        <v>1</v>
       </c>
       <c r="P2" s="2">
-        <f>IF(E2&lt;=70, 0, IF(E2&lt;=80, (E2-70)/(80-70), 1))</f>
-        <v>0.9</v>
+        <f>IF(J9&lt;=70, 0, IF(J9&lt;=80, (J9-70)/(80-70), 1))</f>
+        <v>0</v>
       </c>
       <c r="Q2" s="2" t="str">
         <f>IF(AND(N2&gt;=O2,N2&gt;=P2),"Kering",IF(O2&gt;=P2,"Lembab","Basah"))</f>
-        <v>Basah</v>
+        <v>Lembab</v>
       </c>
       <c r="R2" s="3">
         <f>L2</f>
-        <v>9.9999999999999645E-2</v>
+        <v>0</v>
       </c>
       <c r="S2" s="3">
         <f>MAX(N2, MIN(O2, L2))</f>
-        <v>9.9999999999999645E-2</v>
+        <v>0</v>
       </c>
       <c r="T2" s="3">
         <f>F2</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U2" s="2" t="str">
         <f>IF(R2&gt;0.5,"ON","OFF")</f>
@@ -701,367 +694,557 @@
       </c>
       <c r="W2" s="2" t="str">
         <f>IF(T2&gt;0.4,"ON","OFF")</f>
-        <v>ON</v>
-      </c>
-    </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" s="2">
-        <v>5</v>
-      </c>
-      <c r="D3" s="2">
-        <v>27.5</v>
-      </c>
-      <c r="E3" s="2">
-        <v>79</v>
-      </c>
+        <v>OFF</v>
+      </c>
+    </row>
+    <row r="3" spans="6:23" x14ac:dyDescent="0.25">
       <c r="F3" s="3">
-        <f t="shared" ref="F3:F6" si="0">IF(C3&lt;=5, 1, IF(C3&lt;=6, (6-C3)/(6-5), 0))</f>
+        <f>IF(H10&lt;=5, 1, IF(H10&lt;=6, (6-H10)/(6-5), 0))</f>
+        <v>0</v>
+      </c>
+      <c r="G3" s="2">
+        <f>IF(H10&lt;=5.5, 0, IF(H10&lt;=6, (H10-5.5)/(6-5.5),IF(H10&lt;=7, 1, IF(H10&lt;=7.5, (7.5-H10)/(7.5-7), 0))))</f>
         <v>1</v>
       </c>
-      <c r="G3" s="2">
-        <f t="shared" ref="G3:G6" si="1">IF(C3&lt;=5.5, 0, IF(C3&lt;=6, (C3-5.5)/(6-5.5),IF(C3&lt;=7, 1, IF(C3&lt;=7.5, (7.5-C3)/(7.5-7), 0))))</f>
-        <v>0</v>
-      </c>
       <c r="H3" s="2">
-        <f t="shared" ref="H3:H6" si="2">IF(C3&lt;=7, 0, IF(C3&lt;=7.5, (C3-7)/(7.5-7), 1))</f>
+        <f>IF(H10&lt;=7, 0, IF(H10&lt;=7.5, (H10-7)/(7.5-7), 1))</f>
         <v>0</v>
       </c>
       <c r="I3" s="2" t="str">
-        <f t="shared" ref="I3:I6" si="3">IF(AND(F3&gt;=G3,F3&gt;=H3),"Asam",IF(G3&gt;=H3,"Normal","Basa"))</f>
-        <v>Asam</v>
+        <f t="shared" ref="I3:I6" si="0">IF(AND(F3&gt;=G3,F3&gt;=H3),"Asam",IF(G3&gt;=H3,"Normal","Basa"))</f>
+        <v>Normal</v>
       </c>
       <c r="J3" s="2">
-        <f>IF(D3&lt;=24, 1, IF(D3&lt;=27, (27-D3)/(27-24), 0))</f>
-        <v>0</v>
+        <f>IF(I10&lt;=24, 1, IF(I10&lt;=27, (27-I10)/(27-24), 0))</f>
+        <v>1</v>
       </c>
       <c r="K3" s="3">
-        <f>IF(D3&lt;=27,0,IF(D3&lt;=27,(D3-24)/(27-24),IF(D3&lt;=31,(31-D3)/(31-27),0)))</f>
-        <v>0.875</v>
+        <f>IF(I10&lt;=27,0,IF(I10&lt;=27,(I10-24)/(27-24),IF(I10&lt;=31,(31-I10)/(31-27),0)))</f>
+        <v>0</v>
       </c>
       <c r="L3" s="3">
-        <f>IF(D3&lt;=27, 0, IF(D3&lt;=31, (D3-27)/(31-27), 1))</f>
-        <v>0.125</v>
+        <f>IF(I10&lt;=27, 0, IF(I10&lt;=31, (I10-27)/(31-27), 1))</f>
+        <v>0</v>
       </c>
       <c r="M3" s="2" t="str">
         <f>IF(AND(J3&gt;=K3,J3&gt;=L3),"Rendah",IF(K3&gt;=L3,"Sedang","Tinggi"))</f>
-        <v>Sedang</v>
+        <v>Rendah</v>
       </c>
       <c r="N3" s="2">
-        <f>IF(E3&lt;=40, 1, IF(E3&lt;=50, (50-E3)/(50-40), 0))</f>
+        <f>IF(J10&lt;=40, 1, IF(J10&lt;=50, (50-J10)/(50-40), 0))</f>
         <v>0</v>
       </c>
       <c r="O3" s="3">
-        <f>IF(E3&lt;=40, 0, IF(E3&lt;=50, (E3-40)/(50-40),IF(E3&lt;=70, 1, IF(E3&lt;=80, (80-E3)/(80-70), 0))))</f>
+        <f>IF(J10&lt;=40, 0, IF(J10&lt;=50, (J10-40)/(50-40),IF(J10&lt;=70, 1, IF(J10&lt;=80, (80-J10)/(80-70), 0))))</f>
+        <v>0.9</v>
+      </c>
+      <c r="P3" s="2">
+        <f>IF(J10&lt;=70, 0, IF(J10&lt;=80, (J10-70)/(80-70), 1))</f>
         <v>0.1</v>
-      </c>
-      <c r="P3" s="2">
-        <f>IF(E3&lt;=70, 0, IF(E3&lt;=80, (E3-70)/(80-70), 1))</f>
-        <v>0.9</v>
       </c>
       <c r="Q3" s="2" t="str">
         <f>IF(AND(N3&gt;=O3,N3&gt;=P3),"Kering",IF(O3&gt;=P3,"Lembab","Basah"))</f>
-        <v>Basah</v>
+        <v>Lembab</v>
       </c>
       <c r="R3" s="3">
         <f>L3</f>
-        <v>0.125</v>
+        <v>0</v>
       </c>
       <c r="S3" s="3">
         <f>MAX(N3, MIN(O3, L3))</f>
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="T3" s="3">
-        <f t="shared" ref="T3:T6" si="4">F3</f>
+        <f t="shared" ref="T3:T6" si="1">F3</f>
+        <v>0</v>
+      </c>
+      <c r="U3" s="2" t="str">
+        <f t="shared" ref="U3:U6" si="2">IF(R3&gt;0.5,"ON","OFF")</f>
+        <v>OFF</v>
+      </c>
+      <c r="V3" s="2" t="str">
+        <f t="shared" ref="V3:V6" si="3">IF(S3&gt;0.4,"ON","OFF")</f>
+        <v>OFF</v>
+      </c>
+      <c r="W3" s="2" t="str">
+        <f t="shared" ref="W3:W6" si="4">IF(T3&gt;0.4,"ON","OFF")</f>
+        <v>OFF</v>
+      </c>
+    </row>
+    <row r="4" spans="6:23" x14ac:dyDescent="0.25">
+      <c r="F4" s="3">
+        <f>IF(H11&lt;=5, 1, IF(H11&lt;=6, (6-H11)/(6-5), 0))</f>
+        <v>0</v>
+      </c>
+      <c r="G4" s="2">
+        <f>IF(H11&lt;=5.5, 0, IF(H11&lt;=6, (H11-5.5)/(6-5.5),IF(H11&lt;=7, 1, IF(H11&lt;=7.5, (7.5-H11)/(7.5-7), 0))))</f>
         <v>1</v>
       </c>
-      <c r="U3" s="2" t="str">
-        <f t="shared" ref="U3:U6" si="5">IF(R3&gt;0.5,"ON","OFF")</f>
-        <v>OFF</v>
-      </c>
-      <c r="V3" s="2" t="str">
-        <f t="shared" ref="V3:V6" si="6">IF(S3&gt;0.4,"ON","OFF")</f>
-        <v>OFF</v>
-      </c>
-      <c r="W3" s="2" t="str">
-        <f t="shared" ref="W3:W6" si="7">IF(T3&gt;0.4,"ON","OFF")</f>
-        <v>ON</v>
-      </c>
-    </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" s="2">
-        <v>5</v>
-      </c>
-      <c r="D4" s="2">
-        <v>27.5</v>
-      </c>
-      <c r="E4" s="2">
-        <v>78</v>
-      </c>
-      <c r="F4" s="3">
+      <c r="H4" s="2">
+        <f>IF(H11&lt;=7, 0, IF(H11&lt;=7.5, (H11-7)/(7.5-7), 1))</f>
+        <v>0</v>
+      </c>
+      <c r="I4" s="2" t="str">
         <f t="shared" si="0"/>
+        <v>Normal</v>
+      </c>
+      <c r="J4" s="2">
+        <f>IF(I11&lt;=24, 1, IF(I11&lt;=27, (27-I11)/(27-24), 0))</f>
         <v>1</v>
       </c>
-      <c r="G4" s="2">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H4" s="2">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I4" s="2" t="str">
-        <f t="shared" si="3"/>
-        <v>Asam</v>
-      </c>
-      <c r="J4" s="2">
-        <f>IF(D4&lt;=24, 1, IF(D4&lt;=27, (27-D4)/(27-24), 0))</f>
-        <v>0</v>
-      </c>
       <c r="K4" s="3">
-        <f>IF(D4&lt;=27,0,IF(D4&lt;=27,(D4-24)/(27-24),IF(D4&lt;=31,(31-D4)/(31-27),0)))</f>
-        <v>0.875</v>
+        <f>IF(I11&lt;=27,0,IF(I11&lt;=27,(I11-24)/(27-24),IF(I11&lt;=31,(31-I11)/(31-27),0)))</f>
+        <v>0</v>
       </c>
       <c r="L4" s="3">
-        <f>IF(D4&lt;=27, 0, IF(D4&lt;=31, (D4-27)/(31-27), 1))</f>
-        <v>0.125</v>
+        <f>IF(I11&lt;=27, 0, IF(I11&lt;=31, (I11-27)/(31-27), 1))</f>
+        <v>0</v>
       </c>
       <c r="M4" s="2" t="str">
         <f>IF(AND(J4&gt;=K4,J4&gt;=L4),"Rendah",IF(K4&gt;=L4,"Sedang","Tinggi"))</f>
-        <v>Sedang</v>
+        <v>Rendah</v>
       </c>
       <c r="N4" s="2">
-        <f>IF(E4&lt;=40, 1, IF(E4&lt;=50, (50-E4)/(50-40), 0))</f>
+        <f>IF(J11&lt;=40, 1, IF(J11&lt;=50, (50-J11)/(50-40), 0))</f>
         <v>0</v>
       </c>
       <c r="O4" s="3">
-        <f>IF(E4&lt;=40, 0, IF(E4&lt;=50, (E4-40)/(50-40),IF(E4&lt;=70, 1, IF(E4&lt;=80, (80-E4)/(80-70), 0))))</f>
-        <v>0.2</v>
+        <f>IF(J11&lt;=40, 0, IF(J11&lt;=50, (J11-40)/(50-40),IF(J11&lt;=70, 1, IF(J11&lt;=80, (80-J11)/(80-70), 0))))</f>
+        <v>1</v>
       </c>
       <c r="P4" s="2">
-        <f>IF(E4&lt;=70, 0, IF(E4&lt;=80, (E4-70)/(80-70), 1))</f>
-        <v>0.8</v>
+        <f>IF(J11&lt;=70, 0, IF(J11&lt;=80, (J11-70)/(80-70), 1))</f>
+        <v>0</v>
       </c>
       <c r="Q4" s="2" t="str">
         <f>IF(AND(N4&gt;=O4,N4&gt;=P4),"Kering",IF(O4&gt;=P4,"Lembab","Basah"))</f>
-        <v>Basah</v>
+        <v>Lembab</v>
       </c>
       <c r="R4" s="3">
         <f>L4</f>
-        <v>0.125</v>
+        <v>0</v>
       </c>
       <c r="S4" s="3">
         <f>MAX(N4, MIN(O4, L4))</f>
-        <v>0.125</v>
+        <v>0</v>
       </c>
       <c r="T4" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="U4" s="2" t="str">
+        <f t="shared" si="2"/>
+        <v>OFF</v>
+      </c>
+      <c r="V4" s="2" t="str">
+        <f t="shared" si="3"/>
+        <v>OFF</v>
+      </c>
+      <c r="W4" s="2" t="str">
         <f t="shared" si="4"/>
+        <v>OFF</v>
+      </c>
+    </row>
+    <row r="5" spans="6:23" x14ac:dyDescent="0.25">
+      <c r="F5" s="3">
+        <f>IF(H12&lt;=5, 1, IF(H12&lt;=6, (6-H12)/(6-5), 0))</f>
+        <v>0</v>
+      </c>
+      <c r="G5" s="2">
+        <f>IF(H12&lt;=5.5, 0, IF(H12&lt;=6, (H12-5.5)/(6-5.5),IF(H12&lt;=7, 1, IF(H12&lt;=7.5, (7.5-H12)/(7.5-7), 0))))</f>
         <v>1</v>
       </c>
-      <c r="U4" s="2" t="str">
-        <f t="shared" si="5"/>
-        <v>OFF</v>
-      </c>
-      <c r="V4" s="2" t="str">
-        <f t="shared" si="6"/>
-        <v>OFF</v>
-      </c>
-      <c r="W4" s="2" t="str">
-        <f t="shared" si="7"/>
-        <v>ON</v>
-      </c>
-    </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A5" s="2">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="2">
-        <v>5</v>
-      </c>
-      <c r="D5" s="2">
-        <v>27.4</v>
-      </c>
-      <c r="E5" s="2">
-        <v>79</v>
-      </c>
-      <c r="F5" s="3">
+      <c r="H5" s="2">
+        <f>IF(H12&lt;=7, 0, IF(H12&lt;=7.5, (H12-7)/(7.5-7), 1))</f>
+        <v>0</v>
+      </c>
+      <c r="I5" s="2" t="str">
         <f t="shared" si="0"/>
+        <v>Normal</v>
+      </c>
+      <c r="J5" s="2">
+        <f>IF(I12&lt;=24, 1, IF(I12&lt;=27, (27-I12)/(27-24), 0))</f>
         <v>1</v>
       </c>
-      <c r="G5" s="2">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H5" s="2">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I5" s="2" t="str">
-        <f t="shared" si="3"/>
-        <v>Asam</v>
-      </c>
-      <c r="J5" s="2">
-        <f>IF(D5&lt;=24, 1, IF(D5&lt;=27, (27-D5)/(27-24), 0))</f>
-        <v>0</v>
-      </c>
       <c r="K5" s="3">
-        <f>IF(D5&lt;=27,0,IF(D5&lt;=27,(D5-24)/(27-24),IF(D5&lt;=31,(31-D5)/(31-27),0)))</f>
-        <v>0.90000000000000036</v>
+        <f>IF(I12&lt;=27,0,IF(I12&lt;=27,(I12-24)/(27-24),IF(I12&lt;=31,(31-I12)/(31-27),0)))</f>
+        <v>0</v>
       </c>
       <c r="L5" s="3">
-        <f>IF(D5&lt;=27, 0, IF(D5&lt;=31, (D5-27)/(31-27), 1))</f>
-        <v>9.9999999999999645E-2</v>
+        <f>IF(I12&lt;=27, 0, IF(I12&lt;=31, (I12-27)/(31-27), 1))</f>
+        <v>0</v>
       </c>
       <c r="M5" s="2" t="str">
         <f>IF(AND(J5&gt;=K5,J5&gt;=L5),"Rendah",IF(K5&gt;=L5,"Sedang","Tinggi"))</f>
-        <v>Sedang</v>
+        <v>Rendah</v>
       </c>
       <c r="N5" s="2">
-        <f>IF(E5&lt;=40, 1, IF(E5&lt;=50, (50-E5)/(50-40), 0))</f>
+        <f>IF(J12&lt;=40, 1, IF(J12&lt;=50, (50-J12)/(50-40), 0))</f>
         <v>0</v>
       </c>
       <c r="O5" s="3">
-        <f>IF(E5&lt;=40, 0, IF(E5&lt;=50, (E5-40)/(50-40),IF(E5&lt;=70, 1, IF(E5&lt;=80, (80-E5)/(80-70), 0))))</f>
-        <v>0.1</v>
+        <f>IF(J12&lt;=40, 0, IF(J12&lt;=50, (J12-40)/(50-40),IF(J12&lt;=70, 1, IF(J12&lt;=80, (80-J12)/(80-70), 0))))</f>
+        <v>1</v>
       </c>
       <c r="P5" s="2">
-        <f>IF(E5&lt;=70, 0, IF(E5&lt;=80, (E5-70)/(80-70), 1))</f>
-        <v>0.9</v>
+        <f>IF(J12&lt;=70, 0, IF(J12&lt;=80, (J12-70)/(80-70), 1))</f>
+        <v>0</v>
       </c>
       <c r="Q5" s="2" t="str">
         <f>IF(AND(N5&gt;=O5,N5&gt;=P5),"Kering",IF(O5&gt;=P5,"Lembab","Basah"))</f>
-        <v>Basah</v>
+        <v>Lembab</v>
       </c>
       <c r="R5" s="3">
         <f>L5</f>
-        <v>9.9999999999999645E-2</v>
+        <v>0</v>
       </c>
       <c r="S5" s="3">
         <f>MAX(N5, MIN(O5, L5))</f>
-        <v>9.9999999999999645E-2</v>
+        <v>0</v>
       </c>
       <c r="T5" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="U5" s="2" t="str">
+        <f t="shared" si="2"/>
+        <v>OFF</v>
+      </c>
+      <c r="V5" s="2" t="str">
+        <f t="shared" si="3"/>
+        <v>OFF</v>
+      </c>
+      <c r="W5" s="2" t="str">
         <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="U5" s="2" t="str">
-        <f t="shared" si="5"/>
-        <v>OFF</v>
-      </c>
-      <c r="V5" s="2" t="str">
-        <f t="shared" si="6"/>
-        <v>OFF</v>
-      </c>
-      <c r="W5" s="2" t="str">
-        <f t="shared" si="7"/>
-        <v>ON</v>
-      </c>
-    </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A6" s="2">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" s="2">
-        <v>5</v>
-      </c>
-      <c r="D6" s="2">
-        <v>27.2</v>
-      </c>
-      <c r="E6" s="2">
-        <v>79</v>
-      </c>
+        <v>OFF</v>
+      </c>
+    </row>
+    <row r="6" spans="6:23" x14ac:dyDescent="0.25">
       <c r="F6" s="3">
+        <f>IF(H13&lt;=5, 1, IF(H13&lt;=6, (6-H13)/(6-5), 0))</f>
+        <v>4.9999999999999822E-2</v>
+      </c>
+      <c r="G6" s="2">
+        <f>IF(H13&lt;=5.5, 0, IF(H13&lt;=6, (H13-5.5)/(6-5.5),IF(H13&lt;=7, 1, IF(H13&lt;=7.5, (7.5-H13)/(7.5-7), 0))))</f>
+        <v>0.90000000000000036</v>
+      </c>
+      <c r="H6" s="2">
+        <f>IF(H13&lt;=7, 0, IF(H13&lt;=7.5, (H13-7)/(7.5-7), 1))</f>
+        <v>0</v>
+      </c>
+      <c r="I6" s="2" t="str">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="G6" s="2">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H6" s="2">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I6" s="2" t="str">
-        <f t="shared" si="3"/>
-        <v>Asam</v>
-      </c>
-      <c r="J6" s="2">
-        <f>IF(D6&lt;=24, 1, IF(D6&lt;=27, (27-D6)/(27-24), 0))</f>
-        <v>0</v>
+        <v>Normal</v>
+      </c>
+      <c r="J6" s="3">
+        <f>IF(I13&lt;=24, 1, IF(I13&lt;=27, (27-I13)/(27-24), 0))</f>
+        <v>0.86666666666666714</v>
       </c>
       <c r="K6" s="3">
-        <f>IF(D6&lt;=27,0,IF(D6&lt;=27,(D6-24)/(27-24),IF(D6&lt;=31,(31-D6)/(31-27),0)))</f>
-        <v>0.95000000000000018</v>
+        <f>IF(I13&lt;=27,0,IF(I13&lt;=27,(I13-24)/(27-24),IF(I13&lt;=31,(31-I13)/(31-27),0)))</f>
+        <v>0</v>
       </c>
       <c r="L6" s="3">
-        <f>IF(D6&lt;=27, 0, IF(D6&lt;=31, (D6-27)/(31-27), 1))</f>
-        <v>4.9999999999999822E-2</v>
+        <f>IF(I13&lt;=27, 0, IF(I13&lt;=31, (I13-27)/(31-27), 1))</f>
+        <v>0</v>
       </c>
       <c r="M6" s="2" t="str">
         <f>IF(AND(J6&gt;=K6,J6&gt;=L6),"Rendah",IF(K6&gt;=L6,"Sedang","Tinggi"))</f>
-        <v>Sedang</v>
+        <v>Rendah</v>
       </c>
       <c r="N6" s="2">
-        <f>IF(E6&lt;=40, 1, IF(E6&lt;=50, (50-E6)/(50-40), 0))</f>
-        <v>0</v>
+        <f>IF(J13&lt;=40, 1, IF(J13&lt;=50, (50-J13)/(50-40), 0))</f>
+        <v>0.1</v>
       </c>
       <c r="O6" s="3">
-        <f>IF(E6&lt;=40, 0, IF(E6&lt;=50, (E6-40)/(50-40),IF(E6&lt;=70, 1, IF(E6&lt;=80, (80-E6)/(80-70), 0))))</f>
-        <v>0.1</v>
+        <f>IF(J13&lt;=40, 0, IF(J13&lt;=50, (J13-40)/(50-40),IF(J13&lt;=70, 1, IF(J13&lt;=80, (80-J13)/(80-70), 0))))</f>
+        <v>0.9</v>
       </c>
       <c r="P6" s="2">
-        <f>IF(E6&lt;=70, 0, IF(E6&lt;=80, (E6-70)/(80-70), 1))</f>
-        <v>0.9</v>
+        <f>IF(J13&lt;=70, 0, IF(J13&lt;=80, (J13-70)/(80-70), 1))</f>
+        <v>0</v>
       </c>
       <c r="Q6" s="2" t="str">
         <f>IF(AND(N6&gt;=O6,N6&gt;=P6),"Kering",IF(O6&gt;=P6,"Lembab","Basah"))</f>
-        <v>Basah</v>
+        <v>Lembab</v>
       </c>
       <c r="R6" s="3">
         <f>L6</f>
-        <v>4.9999999999999822E-2</v>
+        <v>0</v>
       </c>
       <c r="S6" s="3">
         <f>MAX(N6, MIN(O6, L6))</f>
+        <v>0.1</v>
+      </c>
+      <c r="T6" s="3">
+        <f t="shared" si="1"/>
         <v>4.9999999999999822E-2</v>
       </c>
-      <c r="T6" s="3">
+      <c r="U6" s="2" t="str">
+        <f t="shared" si="2"/>
+        <v>OFF</v>
+      </c>
+      <c r="V6" s="2" t="str">
+        <f t="shared" si="3"/>
+        <v>OFF</v>
+      </c>
+      <c r="W6" s="2" t="str">
         <f t="shared" si="4"/>
+        <v>OFF</v>
+      </c>
+    </row>
+    <row r="8" spans="6:23" x14ac:dyDescent="0.25">
+      <c r="F8" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="G8" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="U6" s="2" t="str">
-        <f t="shared" si="5"/>
-        <v>OFF</v>
-      </c>
-      <c r="V6" s="2" t="str">
-        <f t="shared" si="6"/>
-        <v>OFF</v>
-      </c>
-      <c r="W6" s="2" t="str">
-        <f t="shared" si="7"/>
-        <v>ON</v>
+      <c r="H8" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="M8" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="N8" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="O8" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="P8" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q8" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="6:23" x14ac:dyDescent="0.25">
+      <c r="F9" s="2">
+        <v>1</v>
+      </c>
+      <c r="G9" s="6">
+        <v>46088</v>
+      </c>
+      <c r="H9" s="3">
+        <v>6.9</v>
+      </c>
+      <c r="I9" s="7">
+        <v>22</v>
+      </c>
+      <c r="J9" s="2">
+        <v>70</v>
+      </c>
+      <c r="M9" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="N9" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="O9" s="5">
+        <v>3</v>
+      </c>
+      <c r="P9" s="5">
+        <v>5</v>
+      </c>
+      <c r="Q9" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="6:23" x14ac:dyDescent="0.25">
+      <c r="F10" s="2">
+        <v>2</v>
+      </c>
+      <c r="G10" s="6">
+        <v>46088</v>
+      </c>
+      <c r="H10" s="3">
+        <v>6.9</v>
+      </c>
+      <c r="I10" s="7">
+        <v>22</v>
+      </c>
+      <c r="J10" s="2">
+        <v>71</v>
+      </c>
+      <c r="M10" s="4"/>
+      <c r="N10" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="O10" s="5">
+        <v>5.5</v>
+      </c>
+      <c r="P10" s="5">
+        <v>6.5</v>
+      </c>
+      <c r="Q10" s="5">
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="11" spans="6:23" x14ac:dyDescent="0.25">
+      <c r="F11" s="2">
+        <v>3</v>
+      </c>
+      <c r="G11" s="6">
+        <v>46119</v>
+      </c>
+      <c r="H11" s="2">
+        <v>6.43</v>
+      </c>
+      <c r="I11" s="2">
+        <v>23.1</v>
+      </c>
+      <c r="J11" s="2">
+        <v>58</v>
+      </c>
+      <c r="M11" s="4"/>
+      <c r="N11" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="O11" s="5">
+        <v>7</v>
+      </c>
+      <c r="P11" s="5">
+        <v>7.5</v>
+      </c>
+      <c r="Q11" s="5">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="6:23" x14ac:dyDescent="0.25">
+      <c r="F12" s="2">
+        <v>4</v>
+      </c>
+      <c r="G12" s="6">
+        <v>46119</v>
+      </c>
+      <c r="H12" s="2">
+        <v>6.31</v>
+      </c>
+      <c r="I12" s="2">
+        <v>23.1</v>
+      </c>
+      <c r="J12" s="2">
+        <v>58</v>
+      </c>
+      <c r="M12" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="N12" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="O12" s="5">
+        <v>0</v>
+      </c>
+      <c r="P12" s="5">
+        <v>24</v>
+      </c>
+      <c r="Q12" s="5">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="6:23" x14ac:dyDescent="0.25">
+      <c r="F13" s="2">
+        <v>5</v>
+      </c>
+      <c r="G13" s="6">
+        <v>46149</v>
+      </c>
+      <c r="H13" s="2">
+        <v>5.95</v>
+      </c>
+      <c r="I13" s="2">
+        <v>24.4</v>
+      </c>
+      <c r="J13" s="2">
+        <v>49</v>
+      </c>
+      <c r="M13" s="4"/>
+      <c r="N13" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="O13" s="5">
+        <v>24</v>
+      </c>
+      <c r="P13" s="5">
+        <v>27</v>
+      </c>
+      <c r="Q13" s="5">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="6:23" x14ac:dyDescent="0.25">
+      <c r="M14" s="4"/>
+      <c r="N14" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="O14" s="5">
+        <v>27</v>
+      </c>
+      <c r="P14" s="5">
+        <v>31</v>
+      </c>
+      <c r="Q14" s="5">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="15" spans="6:23" x14ac:dyDescent="0.25">
+      <c r="M15" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="N15" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="O15" s="5">
+        <v>0</v>
+      </c>
+      <c r="P15" s="5">
+        <v>40</v>
+      </c>
+      <c r="Q15" s="5">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="16" spans="6:23" x14ac:dyDescent="0.25">
+      <c r="M16" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="N16" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="O16" s="5">
+        <v>40</v>
+      </c>
+      <c r="P16" s="5">
+        <v>60</v>
+      </c>
+      <c r="Q16" s="5">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="17" spans="13:17" x14ac:dyDescent="0.25">
+      <c r="M17" s="4"/>
+      <c r="N17" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="O17" s="5">
+        <v>70</v>
+      </c>
+      <c r="P17" s="5">
+        <v>80</v>
+      </c>
+      <c r="Q17" s="5">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup scale="69" orientation="landscape" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <pageSetup scale="66" orientation="landscape" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>